<commit_message>
Enhance vaccine campaign deduplication logic to include checks for HQ initiated campaigns and existing customer bookings, ensuring appropriate manual review flags. Update import functionality to handle acknowledgment and carepro clinic assignments, improving data integrity during campaign imports. Modify .gitignore to include backup directory.
</commit_message>
<xml_diff>
--- a/vaccine_campaign_template.xlsx
+++ b/vaccine_campaign_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\odb\blood_test\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\odb\vaccination\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6B2838E-EDB1-4A19-B695-1D3A522B63B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13D78425-5A4B-4FE9-BB18-D5C3499240A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9252" yWindow="3756" windowWidth="16056" windowHeight="7764" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="37650" yWindow="6450" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Date</t>
   </si>
@@ -37,18 +37,30 @@
   </si>
   <si>
     <t>&lt;--Please do not delete this row</t>
+  </si>
+  <si>
+    <t>Acknowledge</t>
+  </si>
+  <si>
+    <t>Carepro Mobile Clinic</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -69,10 +81,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -80,9 +93,13 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{5BDFA75A-C69A-4B29-8BF3-EBB6E148624C}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -360,29 +377,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="3"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>45954</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>